<commit_message>
Add Supabase integration, GitHub Actions CI, and database migrations
- Add dual storage mode (Excel + Supabase) to scraper
- Create Supabase migrations for properties and availability tables
- Set up GitHub Actions workflow for twice-daily automated scraping
- Add seed script for migrating Excel data to Supabase
- Add .gitignore for .env, __pycache__, and debug HTML files
- Add supabase==2.28.0 to requirements
</commit_message>
<xml_diff>
--- a/KuceZaIzdavanje.xlsx
+++ b/KuceZaIzdavanje.xlsx
@@ -28246,7 +28246,7 @@
       </c>
       <c r="D922" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E922" s="0" t="inlineStr">
@@ -28274,7 +28274,7 @@
       </c>
       <c r="D923" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E923" s="0" t="inlineStr">
@@ -28302,7 +28302,7 @@
       </c>
       <c r="D924" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E924" s="0" t="inlineStr">
@@ -28330,7 +28330,7 @@
       </c>
       <c r="D925" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E925" s="0" t="inlineStr">
@@ -28358,7 +28358,7 @@
       </c>
       <c r="D926" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E926" s="0" t="inlineStr">
@@ -28386,7 +28386,7 @@
       </c>
       <c r="D927" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E927" s="0" t="inlineStr">
@@ -28414,7 +28414,7 @@
       </c>
       <c r="D928" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E928" s="0" t="inlineStr">
@@ -28442,7 +28442,7 @@
       </c>
       <c r="D929" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E929" s="0" t="inlineStr">
@@ -28470,7 +28470,7 @@
       </c>
       <c r="D930" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E930" s="0" t="inlineStr">
@@ -28498,7 +28498,7 @@
       </c>
       <c r="D931" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E931" s="0" t="inlineStr">
@@ -28526,7 +28526,7 @@
       </c>
       <c r="D932" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E932" s="0" t="inlineStr">
@@ -28554,7 +28554,7 @@
       </c>
       <c r="D933" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E933" s="0" t="inlineStr">
@@ -28582,7 +28582,7 @@
       </c>
       <c r="D934" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E934" s="0" t="inlineStr">
@@ -28610,7 +28610,7 @@
       </c>
       <c r="D935" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E935" s="0" t="inlineStr">
@@ -28638,7 +28638,7 @@
       </c>
       <c r="D936" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E936" s="0" t="inlineStr">
@@ -28666,7 +28666,7 @@
       </c>
       <c r="D937" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E937" s="0" t="inlineStr">
@@ -28694,7 +28694,7 @@
       </c>
       <c r="D938" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E938" s="0" t="inlineStr">
@@ -28722,7 +28722,7 @@
       </c>
       <c r="D939" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E939" s="0" t="inlineStr">
@@ -28750,7 +28750,7 @@
       </c>
       <c r="D940" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E940" s="0" t="inlineStr">
@@ -28778,7 +28778,7 @@
       </c>
       <c r="D941" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E941" s="0" t="inlineStr">
@@ -28806,7 +28806,7 @@
       </c>
       <c r="D942" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E942" s="0" t="inlineStr">
@@ -28834,7 +28834,7 @@
       </c>
       <c r="D943" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E943" s="0" t="inlineStr">
@@ -28862,7 +28862,7 @@
       </c>
       <c r="D944" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E944" s="0" t="inlineStr">
@@ -28890,7 +28890,7 @@
       </c>
       <c r="D945" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E945" s="0" t="inlineStr">
@@ -28918,7 +28918,7 @@
       </c>
       <c r="D946" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E946" s="0" t="inlineStr">
@@ -28946,7 +28946,7 @@
       </c>
       <c r="D947" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E947" s="0" t="inlineStr">
@@ -28974,7 +28974,7 @@
       </c>
       <c r="D948" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E948" s="0" t="inlineStr">
@@ -29002,7 +29002,7 @@
       </c>
       <c r="D949" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E949" s="0" t="inlineStr">
@@ -29030,7 +29030,7 @@
       </c>
       <c r="D950" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E950" s="0" t="inlineStr">
@@ -29058,7 +29058,7 @@
       </c>
       <c r="D951" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E951" s="0" t="inlineStr">
@@ -29086,7 +29086,7 @@
       </c>
       <c r="D952" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E952" s="0" t="inlineStr">
@@ -29114,7 +29114,7 @@
       </c>
       <c r="D953" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E953" s="0" t="inlineStr">
@@ -29142,7 +29142,7 @@
       </c>
       <c r="D954" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E954" s="0" t="inlineStr">
@@ -29170,7 +29170,7 @@
       </c>
       <c r="D955" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E955" s="0" t="inlineStr">
@@ -29198,7 +29198,7 @@
       </c>
       <c r="D956" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E956" s="0" t="inlineStr">
@@ -29226,7 +29226,7 @@
       </c>
       <c r="D957" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E957" s="0" t="inlineStr">
@@ -29254,7 +29254,7 @@
       </c>
       <c r="D958" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E958" s="0" t="inlineStr">
@@ -29282,7 +29282,7 @@
       </c>
       <c r="D959" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E959" s="0" t="inlineStr">
@@ -29310,7 +29310,7 @@
       </c>
       <c r="D960" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E960" s="0" t="inlineStr">
@@ -29338,7 +29338,7 @@
       </c>
       <c r="D961" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E961" s="0" t="inlineStr">
@@ -29366,7 +29366,7 @@
       </c>
       <c r="D962" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E962" s="0" t="inlineStr">
@@ -29394,7 +29394,7 @@
       </c>
       <c r="D963" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E963" s="0" t="inlineStr">
@@ -29422,7 +29422,7 @@
       </c>
       <c r="D964" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E964" s="0" t="inlineStr">
@@ -29450,7 +29450,7 @@
       </c>
       <c r="D965" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E965" s="0" t="inlineStr">
@@ -29478,7 +29478,7 @@
       </c>
       <c r="D966" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E966" s="0" t="inlineStr">
@@ -29506,7 +29506,7 @@
       </c>
       <c r="D967" s="0" t="inlineStr">
         <is>
-          <t>2026-03-01 09:45:30</t>
+          <t>2026-03-01 10:29:28</t>
         </is>
       </c>
       <c r="E967" s="0" t="inlineStr">

</xml_diff>